<commit_message>
智康保 额度申请 71 72  88 95 96  145  146
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/zkb/contract/excel/APM_ZKB_Contract_imp_Template.xlsx
+++ b/src/src/main/webapp/portal/zkb/contract/excel/APM_ZKB_Contract_imp_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Intellij Idea\codes\hc-apm-web\src\src\main\webapp\portal\zkb\contract\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498F5AE7-90BA-423F-8869-6F3141D7DD7D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B301C6FB-84CD-413C-B0D2-08538BA62CD8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1155" windowWidth="29040" windowHeight="15840" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
   </bookViews>
   <sheets>
     <sheet name="合同" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
   <si>
     <t>代理商</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>备件+人工+保养已使用名额</t>
+  </si>
+  <si>
+    <t>备注</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -204,6 +207,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,28 +532,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C52200B-3B0C-4F93-BC6C-7CAE122E49C2}">
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.21875" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" customWidth="1"/>
-    <col min="13" max="13" width="17.21875" customWidth="1"/>
-    <col min="14" max="14" width="16.77734375" customWidth="1"/>
-    <col min="15" max="15" width="19.44140625" customWidth="1"/>
-    <col min="16" max="16" width="21.44140625" customWidth="1"/>
-    <col min="17" max="17" width="23.21875" customWidth="1"/>
-    <col min="18" max="18" width="26.5546875" customWidth="1"/>
-    <col min="19" max="19" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="19.42578125" customWidth="1"/>
+    <col min="16" max="16" width="21.42578125" customWidth="1"/>
+    <col min="17" max="17" width="23.28515625" customWidth="1"/>
+    <col min="18" max="18" width="26.5703125" customWidth="1"/>
+    <col min="19" max="19" width="29.140625" customWidth="1"/>
+    <col min="20" max="20" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="4" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
@@ -553,10 +567,10 @@
       <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="9" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
@@ -598,6 +612,12 @@
       <c r="S1" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="T1" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="E12" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -608,16 +628,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD4DBF4-FEF1-4385-BAD9-BD07A4FA541B}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
@@ -647,19 +667,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEEB4E3A-F934-494E-85E2-577CC5C4A5F0}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="7.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="7.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
-    <col min="8" max="8" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>

</xml_diff>